<commit_message>
Daily local update (bizportal/BOI blocked from GitHub)
</commit_message>
<xml_diff>
--- a/ytm_computed.xlsx
+++ b/ytm_computed.xlsx
@@ -943,22 +943,22 @@
         <v>1082</v>
       </c>
       <c r="AY2" s="11" t="n">
-        <v>0.08268320268530761</v>
+        <v>0.08271512196505244</v>
       </c>
       <c r="AZ2" s="12" t="n">
         <v>0.6749418153607452</v>
       </c>
       <c r="BA2" s="8" t="n">
-        <v>3.038208683697854</v>
+        <v>3.035452709918621</v>
       </c>
       <c r="BB2" s="8" t="n">
-        <v>2.806184372457599</v>
+        <v>2.80355621560867</v>
       </c>
       <c r="BC2" s="8" t="n">
-        <v>3.273972602739726</v>
+        <v>3.271232876712329</v>
       </c>
       <c r="BD2" s="11" t="n">
-        <v>0.003291413145402782</v>
+        <v>0.003294401512935477</v>
       </c>
       <c r="BE2" s="1" t="n"/>
       <c r="BF2" s="1" t="n"/>
@@ -1040,7 +1040,7 @@
         <v>97.62132</v>
       </c>
       <c r="AJ3" t="n">
-        <v>9823</v>
+        <v>9737</v>
       </c>
       <c r="AK3" s="10" t="n">
         <v>46924</v>
@@ -1054,22 +1054,22 @@
         <v>1036</v>
       </c>
       <c r="AY3" s="11" t="n">
-        <v>-0.009236975335859465</v>
+        <v>-0.009318928716467676</v>
       </c>
       <c r="AZ3" s="12" t="n">
-        <v>0.09815289219179468</v>
+        <v>0.1078520961281708</v>
       </c>
       <c r="BA3" s="8" t="n">
-        <v>1.750699546841039</v>
+        <v>1.747963286746559</v>
       </c>
       <c r="BB3" s="8" t="n">
-        <v>1.767021480675977</v>
+        <v>1.764405657293812</v>
       </c>
       <c r="BC3" s="8" t="n">
-        <v>1.76986301369863</v>
+        <v>1.767123287671233</v>
       </c>
       <c r="BD3" s="11" t="n">
-        <v>0.005712002392440208</v>
+        <v>0.005720943955643803</v>
       </c>
     </row>
     <row r="4">
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>113</v>
+        <v>113.2</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -1163,22 +1163,22 @@
         <v>1978</v>
       </c>
       <c r="AY4" s="11" t="n">
-        <v>0.01748300266381058</v>
+        <v>0.01706306207265681</v>
       </c>
       <c r="AZ4" s="12" t="n">
-        <v>0.1917137476459512</v>
+        <v>0.1938229755178908</v>
       </c>
       <c r="BA4" s="8" t="n">
-        <v>4.403122072273234</v>
+        <v>4.400806383572784</v>
       </c>
       <c r="BB4" s="8" t="n">
-        <v>4.327464990319924</v>
+        <v>4.326974941558146</v>
       </c>
       <c r="BC4" s="8" t="n">
-        <v>4.76986301369863</v>
+        <v>4.767123287671233</v>
       </c>
       <c r="BD4" s="11" t="n">
-        <v>0.002271115775547241</v>
+        <v>0.00227231082860808</v>
       </c>
     </row>
     <row r="5">
@@ -1258,7 +1258,7 @@
         <v>165</v>
       </c>
       <c r="AJ5" t="n">
-        <v>6149</v>
+        <v>6148</v>
       </c>
       <c r="AK5" s="10" t="n">
         <v>46377</v>
@@ -1272,22 +1272,22 @@
         <v>2101</v>
       </c>
       <c r="AY5" s="11" t="n">
-        <v>0.04216221893268751</v>
+        <v>0.04244003775595155</v>
       </c>
       <c r="AZ5" s="12" t="n">
-        <v>1.659212880143112</v>
+        <v>1.659645413142485</v>
       </c>
       <c r="BA5" s="8" t="n">
-        <v>0.2986301369863014</v>
+        <v>0.2958904109589041</v>
       </c>
       <c r="BB5" s="8" t="n">
-        <v>0.2865486116855572</v>
+        <v>0.2838440584034588</v>
       </c>
       <c r="BC5" s="8" t="n">
-        <v>0.2712328767123288</v>
+        <v>0.2684931506849315</v>
       </c>
       <c r="BD5" s="11" t="n">
-        <v>0.03348623853211009</v>
+        <v>0.0337962962962963</v>
       </c>
     </row>
     <row r="6">
@@ -1385,7 +1385,7 @@
         <v>80</v>
       </c>
       <c r="AJ6" t="n">
-        <v>22500</v>
+        <v>22120</v>
       </c>
       <c r="AK6" s="10" t="n">
         <v>48813</v>
@@ -1399,22 +1399,22 @@
         <v>720</v>
       </c>
       <c r="AY6" s="11" t="n">
-        <v>-0.1187210331918223</v>
+        <v>-0.1187727106458985</v>
       </c>
       <c r="AZ6" s="12" t="n">
-        <v>0.02684444444444445</v>
+        <v>0.04448462929475583</v>
       </c>
       <c r="BA6" s="8" t="n">
-        <v>6.554061623195342</v>
+        <v>6.551409702638343</v>
       </c>
       <c r="BB6" s="8" t="n">
-        <v>7.436988592764092</v>
+        <v>7.434415367958272</v>
       </c>
       <c r="BC6" s="8" t="n">
-        <v>6.945205479452055</v>
+        <v>6.942465753424657</v>
       </c>
       <c r="BD6" s="11" t="n">
-        <v>0.00152577143379446</v>
+        <v>0.001526389045089466</v>
       </c>
     </row>
     <row r="7">
@@ -1494,7 +1494,7 @@
         <v>240</v>
       </c>
       <c r="AJ7" t="n">
-        <v>22500</v>
+        <v>22120</v>
       </c>
       <c r="AK7" s="10" t="n">
         <v>46987</v>
@@ -1508,22 +1508,22 @@
         <v>720</v>
       </c>
       <c r="AY7" s="11" t="n">
-        <v>-0.05974016890131063</v>
+        <v>-0.05982984961643226</v>
       </c>
       <c r="AZ7" s="12" t="n">
-        <v>0.2213333333333334</v>
+        <v>0.2423146473779385</v>
       </c>
       <c r="BA7" s="8" t="n">
-        <v>1.960172486638279</v>
+        <v>1.957433418961262</v>
       </c>
       <c r="BB7" s="8" t="n">
-        <v>2.084713631069219</v>
+        <v>2.081999112780462</v>
       </c>
       <c r="BC7" s="8" t="n">
-        <v>1.942465753424657</v>
+        <v>1.93972602739726</v>
       </c>
       <c r="BD7" s="11" t="n">
-        <v>0.005101591858964477</v>
+        <v>0.005108730597491604</v>
       </c>
     </row>
     <row r="8">
@@ -1603,7 +1603,7 @@
         <v>84.29154</v>
       </c>
       <c r="AJ8" t="n">
-        <v>2012</v>
+        <v>1956</v>
       </c>
       <c r="AK8" s="10" t="n">
         <v>46590</v>
@@ -1617,22 +1617,22 @@
         <v>1581</v>
       </c>
       <c r="AY8" s="11" t="n">
-        <v>0.04369020246746916</v>
+        <v>0.04381792993224948</v>
       </c>
       <c r="AZ8" s="12" t="n">
-        <v>3.042809945328032</v>
+        <v>3.158555015337424</v>
       </c>
       <c r="BA8" s="8" t="n">
-        <v>0.8821917808219178</v>
+        <v>0.8794520547945205</v>
       </c>
       <c r="BB8" s="8" t="n">
-        <v>0.8452621081775603</v>
+        <v>0.842533960737389</v>
       </c>
       <c r="BC8" s="8" t="n">
-        <v>0.8547945205479452</v>
+        <v>0.852054794520548</v>
       </c>
       <c r="BD8" s="11" t="n">
-        <v>0.01133540372670807</v>
+        <v>0.01137071651090343</v>
       </c>
     </row>
     <row r="9">
@@ -1712,7 +1712,7 @@
         <v>9.529999999999999</v>
       </c>
       <c r="AJ9" t="n">
-        <v>246.3</v>
+        <v>250</v>
       </c>
       <c r="AK9" s="10" t="n">
         <v>46895</v>
@@ -1729,22 +1729,22 @@
         <v>1975</v>
       </c>
       <c r="AY9" s="11" t="n">
-        <v>0.1532527088191327</v>
+        <v>0.1534238980651479</v>
       </c>
       <c r="AZ9" s="12" t="n">
-        <v>2.277267559886317</v>
+        <v>2.228764</v>
       </c>
       <c r="BA9" s="8" t="n">
-        <v>1.661960930217891</v>
+        <v>1.659214471031818</v>
       </c>
       <c r="BB9" s="8" t="n">
-        <v>1.441107328435974</v>
+        <v>1.438512305679747</v>
       </c>
       <c r="BC9" s="8" t="n">
-        <v>1.69041095890411</v>
+        <v>1.687671232876712</v>
       </c>
       <c r="BD9" s="11" t="n">
-        <v>0.006016988617589798</v>
+        <v>0.006026948399130878</v>
       </c>
     </row>
     <row r="10">
@@ -1845,7 +1845,7 @@
         <v>160</v>
       </c>
       <c r="AJ10" t="n">
-        <v>12720</v>
+        <v>12650</v>
       </c>
       <c r="AK10" s="10" t="n">
         <v>47840</v>
@@ -1859,22 +1859,22 @@
         <v>1884</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>-0.0113631438252168</v>
+        <v>-0.0113820607997417</v>
       </c>
       <c r="AZ10" s="3" t="n">
-        <v>0.4327044025157232</v>
+        <v>0.4406324110671938</v>
       </c>
       <c r="BA10" s="4" t="n">
-        <v>4.122568733752124</v>
+        <v>4.119838482280837</v>
       </c>
       <c r="BB10" s="4" t="n">
-        <v>4.169952503797093</v>
+        <v>4.167270609729758</v>
       </c>
       <c r="BC10" s="4" t="n">
-        <v>4.279452054794521</v>
+        <v>4.276712328767124</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>0.002425672110237584</v>
+        <v>0.002427279623463241</v>
       </c>
       <c r="BE10" s="1" t="n">
         <v>3.73</v>
@@ -1996,22 +1996,22 @@
         <v>126</v>
       </c>
       <c r="AY11" s="11" t="n">
-        <v>0.03399955114350078</v>
+        <v>0.03398011624199031</v>
       </c>
       <c r="AZ11" s="12" t="n">
         <v>0.4991128765880217</v>
       </c>
       <c r="BA11" s="8" t="n">
-        <v>2.648220398574267</v>
+        <v>2.645484944597639</v>
       </c>
       <c r="BB11" s="8" t="n">
-        <v>2.561142696479508</v>
+        <v>2.558545278619744</v>
       </c>
       <c r="BC11" s="8" t="n">
-        <v>2.76986301369863</v>
+        <v>2.767123287671233</v>
       </c>
       <c r="BD11" s="11" t="n">
-        <v>0.003776120750895107</v>
+        <v>0.003780025291930336</v>
       </c>
     </row>
     <row r="12">
@@ -2111,7 +2111,7 @@
       <c r="BA12" s="8" t="n"/>
       <c r="BB12" s="8" t="n"/>
       <c r="BC12" s="8" t="n">
-        <v>-0.0547945205479452</v>
+        <v>-0.05753424657534247</v>
       </c>
       <c r="BD12" s="11" t="n"/>
       <c r="BE12" s="1" t="n"/>
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>225</v>
+        <v>222.3</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -2194,7 +2194,7 @@
         <v>1</v>
       </c>
       <c r="AJ13" t="n">
-        <v>220.5</v>
+        <v>219.7</v>
       </c>
       <c r="AK13" s="10" t="n">
         <v>47928</v>
@@ -2208,22 +2208,22 @@
         <v>1006</v>
       </c>
       <c r="AY13" s="11" t="n">
-        <v>-0.1292048653120022</v>
+        <v>-0.1268420572622477</v>
       </c>
       <c r="AZ13" s="12" t="n">
-        <v>0.02040816326530615</v>
+        <v>0.01183431952662728</v>
       </c>
       <c r="BA13" s="8" t="n">
-        <v>4.245477083860979</v>
+        <v>4.240636629461016</v>
       </c>
       <c r="BB13" s="8" t="n">
-        <v>4.875402852798569</v>
+        <v>4.856666156142</v>
       </c>
       <c r="BC13" s="8" t="n">
-        <v>4.52054794520548</v>
+        <v>4.517808219178082</v>
       </c>
       <c r="BD13" s="11" t="n">
-        <v>0.002355447880761063</v>
+        <v>0.002358136495479689</v>
       </c>
     </row>
     <row r="14">
@@ -2303,7 +2303,7 @@
         <v>1.12975</v>
       </c>
       <c r="AJ14" t="n">
-        <v>250</v>
+        <v>249.9</v>
       </c>
       <c r="AK14" s="10" t="n">
         <v>47473</v>
@@ -2317,22 +2317,22 @@
         <v>1769</v>
       </c>
       <c r="AY14" s="11" t="n">
-        <v>-0.1937136919991779</v>
+        <v>-0.1938762443979485</v>
       </c>
       <c r="AZ14" s="12" t="n">
-        <v>0.01632310000000015</v>
+        <v>0.01672979191676682</v>
       </c>
       <c r="BA14" s="8" t="n">
-        <v>3.167146799321049</v>
+        <v>3.164462117537143</v>
       </c>
       <c r="BB14" s="8" t="n">
-        <v>3.928067198826622</v>
+        <v>3.925528922260543</v>
       </c>
       <c r="BC14" s="8" t="n">
-        <v>3.273972602739726</v>
+        <v>3.271232876712329</v>
       </c>
       <c r="BD14" s="11" t="n">
-        <v>0.003157416006780529</v>
+        <v>0.003160094710750673</v>
       </c>
     </row>
     <row r="15">
@@ -2412,7 +2412,7 @@
         <v>0.545</v>
       </c>
       <c r="AJ15" t="n">
-        <v>77.40000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="AK15" s="10" t="n">
         <v>47021</v>
@@ -2426,22 +2426,22 @@
         <v>1532</v>
       </c>
       <c r="AY15" s="11" t="n">
-        <v>-0.1680461872410457</v>
+        <v>-0.1683137203804096</v>
       </c>
       <c r="AZ15" s="12" t="n">
-        <v>0.1611175710594315</v>
+        <v>0.09731990231990229</v>
       </c>
       <c r="BA15" s="8" t="n">
-        <v>1.917472566146698</v>
+        <v>1.914796123587026</v>
       </c>
       <c r="BB15" s="8" t="n">
-        <v>2.304782473185511</v>
+        <v>2.302305773834391</v>
       </c>
       <c r="BC15" s="8" t="n">
-        <v>2.035616438356164</v>
+        <v>2.032876712328767</v>
       </c>
       <c r="BD15" s="11" t="n">
-        <v>0.00521519847352796</v>
+        <v>0.005222488116002031</v>
       </c>
     </row>
     <row r="16">
@@ -2521,7 +2521,7 @@
         <v>187.6184</v>
       </c>
       <c r="AJ16" t="n">
-        <v>18480</v>
+        <v>18390</v>
       </c>
       <c r="AK16" s="10" t="n">
         <v>46924</v>
@@ -2535,22 +2535,22 @@
         <v>767</v>
       </c>
       <c r="AY16" s="11" t="n">
-        <v>-0.03971512311395421</v>
+        <v>-0.03980835140533329</v>
       </c>
       <c r="AZ16" s="12" t="n">
-        <v>0.1401269653679655</v>
+        <v>0.1457067058183796</v>
       </c>
       <c r="BA16" s="8" t="n">
-        <v>1.771634981755567</v>
+        <v>1.768897426707509</v>
       </c>
       <c r="BB16" s="8" t="n">
-        <v>1.844905636232155</v>
+        <v>1.842233713755438</v>
       </c>
       <c r="BC16" s="8" t="n">
-        <v>1.76986301369863</v>
+        <v>1.767123287671233</v>
       </c>
       <c r="BD16" s="11" t="n">
-        <v>0.005644503581708854</v>
+        <v>0.00565323904541669</v>
       </c>
     </row>
     <row r="17">
@@ -2665,22 +2665,22 @@
         <v>486</v>
       </c>
       <c r="AY17" s="11" t="n">
-        <v>0.05568640271019477</v>
+        <v>0.05569127613617968</v>
       </c>
       <c r="AZ17" s="12" t="n">
         <v>0.8535888077858882</v>
       </c>
       <c r="BA17" s="8" t="n">
-        <v>3.018746628596366</v>
+        <v>3.016004211021325</v>
       </c>
       <c r="BB17" s="8" t="n">
-        <v>2.859510760815461</v>
+        <v>2.856899814555514</v>
       </c>
       <c r="BC17" s="8" t="n">
-        <v>3.273972602739726</v>
+        <v>3.271232876712329</v>
       </c>
       <c r="BD17" s="11" t="n">
-        <v>0.003312633099204395</v>
+        <v>0.003315645237979839</v>
       </c>
     </row>
     <row r="18">
@@ -2795,22 +2795,22 @@
         <v>2386</v>
       </c>
       <c r="AY18" s="11" t="n">
-        <v>0.1331597716575706</v>
+        <v>0.1332819046315776</v>
       </c>
       <c r="AZ18" s="12" t="n">
         <v>1.745549738219896</v>
       </c>
       <c r="BA18" s="8" t="n">
-        <v>1.743323168838557</v>
+        <v>1.740578207252948</v>
       </c>
       <c r="BB18" s="8" t="n">
-        <v>1.53846192959043</v>
+        <v>1.535873995816423</v>
       </c>
       <c r="BC18" s="8" t="n">
-        <v>1.76986301369863</v>
+        <v>1.767123287671233</v>
       </c>
       <c r="BD18" s="11" t="n">
-        <v>0.005736171112016044</v>
+        <v>0.005745217283733784</v>
       </c>
     </row>
     <row r="19">
@@ -2890,7 +2890,7 @@
         <v>2.1</v>
       </c>
       <c r="AJ19" t="n">
-        <v>154.3</v>
+        <v>152</v>
       </c>
       <c r="AK19" s="10" t="n">
         <v>47532</v>
@@ -2904,22 +2904,22 @@
         <v>1238</v>
       </c>
       <c r="AY19" s="11" t="n">
-        <v>0.02026932480156678</v>
+        <v>0.02024971190493471</v>
       </c>
       <c r="AZ19" s="12" t="n">
-        <v>0.4834737524303305</v>
+        <v>0.5059210526315789</v>
       </c>
       <c r="BA19" s="8" t="n">
-        <v>3.210498789940575</v>
+        <v>3.207769121268711</v>
       </c>
       <c r="BB19" s="8" t="n">
-        <v>3.146716961783584</v>
+        <v>3.144101962331753</v>
       </c>
       <c r="BC19" s="8" t="n">
-        <v>3.435616438356164</v>
+        <v>3.432876712328767</v>
       </c>
       <c r="BD19" s="11" t="n">
-        <v>0.003114780803323429</v>
+        <v>0.003117431343077734</v>
       </c>
     </row>
     <row r="20">
@@ -2999,7 +2999,7 @@
         <v>80.28818</v>
       </c>
       <c r="AJ20" t="n">
-        <v>27620</v>
+        <v>27690</v>
       </c>
       <c r="AK20" s="10" t="n">
         <v>46801</v>
@@ -3013,22 +3013,22 @@
         <v>224</v>
       </c>
       <c r="AY20" s="11" t="n">
-        <v>-0.5631485611897022</v>
+        <v>-0.5638402332481854</v>
       </c>
       <c r="AZ20" s="12" t="n">
-        <v>0.008979988341781375</v>
+        <v>0.006429298591549282</v>
       </c>
       <c r="BA20" s="8" t="n">
-        <v>1.448515209014694</v>
+        <v>1.445793882197358</v>
       </c>
       <c r="BB20" s="8" t="n">
-        <v>3.315807343932569</v>
+        <v>3.314826337524273</v>
       </c>
       <c r="BC20" s="8" t="n">
-        <v>1.432876712328767</v>
+        <v>1.43013698630137</v>
       </c>
       <c r="BD20" s="11" t="n">
-        <v>0.006903620989110757</v>
+        <v>0.006916615240342363</v>
       </c>
       <c r="BE20" s="1" t="n"/>
       <c r="BF20" s="1" t="n"/>
@@ -3110,7 +3110,7 @@
         <v>6.72026</v>
       </c>
       <c r="AJ21" t="n">
-        <v>475</v>
+        <v>470.3</v>
       </c>
       <c r="AK21" s="10" t="n">
         <v>46559</v>
@@ -3124,22 +3124,22 @@
         <v>473</v>
       </c>
       <c r="AY21" s="11" t="n">
-        <v>0.03830562373296448</v>
+        <v>0.03831046980256778</v>
       </c>
       <c r="AZ21" s="12" t="n">
-        <v>0.4119619957894736</v>
+        <v>0.4260726089729958</v>
       </c>
       <c r="BA21" s="8" t="n">
-        <v>0.7972602739726028</v>
+        <v>0.7945205479452054</v>
       </c>
       <c r="BB21" s="8" t="n">
-        <v>0.767847400369706</v>
+        <v>0.7652051780776915</v>
       </c>
       <c r="BC21" s="8" t="n">
-        <v>0.7698630136986301</v>
+        <v>0.7671232876712328</v>
       </c>
       <c r="BD21" s="11" t="n">
-        <v>0.01254295532646048</v>
+        <v>0.01258620689655172</v>
       </c>
       <c r="BE21" s="1" t="n"/>
       <c r="BF21" s="1" t="n"/>
@@ -3164,7 +3164,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>97.7</v>
+        <v>98</v>
       </c>
       <c r="F22" t="n">
         <v>1.75</v>
@@ -3259,22 +3259,22 @@
         <v>345</v>
       </c>
       <c r="AY22" s="11" t="n">
-        <v>0.08258350038318134</v>
+        <v>0.08092618985831926</v>
       </c>
       <c r="AZ22" s="12" t="n">
-        <v>0.1118753092528451</v>
+        <v>0.1152894606630379</v>
       </c>
       <c r="BA22" s="8" t="n">
-        <v>1.853961480687864</v>
+        <v>1.851666823597571</v>
       </c>
       <c r="BB22" s="8" t="n">
-        <v>1.712534395759452</v>
+        <v>1.713037246178923</v>
       </c>
       <c r="BC22" s="8" t="n">
-        <v>2.035616438356164</v>
+        <v>2.032876712328767</v>
       </c>
       <c r="BD22" s="11" t="n">
-        <v>0.005393855322328359</v>
+        <v>0.005400539596303385</v>
       </c>
     </row>
     <row r="23">
@@ -3354,7 +3354,7 @@
         <v>176.17507</v>
       </c>
       <c r="AJ23" t="n">
-        <v>10630</v>
+        <v>10670</v>
       </c>
       <c r="AK23" s="10" t="n">
         <v>47870</v>
@@ -3368,22 +3368,22 @@
         <v>445</v>
       </c>
       <c r="AY23" s="11" t="n">
-        <v>0.02240400785721699</v>
+        <v>0.02241485666917468</v>
       </c>
       <c r="AZ23" s="12" t="n">
-        <v>0.538010018438382</v>
+        <v>0.5322442826616682</v>
       </c>
       <c r="BA23" s="8" t="n">
-        <v>4.336953443792852</v>
+        <v>4.334212076252138</v>
       </c>
       <c r="BB23" s="8" t="n">
-        <v>4.241917490994935</v>
+        <v>4.239191212823475</v>
       </c>
       <c r="BC23" s="8" t="n">
-        <v>4.361643835616438</v>
+        <v>4.358904109589041</v>
       </c>
       <c r="BD23" s="11" t="n">
-        <v>0.002305766047434111</v>
+        <v>0.002307224432969408</v>
       </c>
     </row>
     <row r="24" customFormat="1" s="1">
@@ -3477,22 +3477,22 @@
         <v>544</v>
       </c>
       <c r="AY24" s="11" t="n">
-        <v>0.1745581673007211</v>
+        <v>0.1746552923326495</v>
       </c>
       <c r="AZ24" s="12" t="n">
         <v>0.4951934058064515</v>
       </c>
       <c r="BA24" s="8" t="n">
-        <v>2.922075572571685</v>
+        <v>2.919272241797438</v>
       </c>
       <c r="BB24" s="8" t="n">
-        <v>2.487808312879875</v>
+        <v>2.48521609773732</v>
       </c>
       <c r="BC24" s="8" t="n">
-        <v>3.273972602739726</v>
+        <v>3.271232876712329</v>
       </c>
       <c r="BD24" s="11" t="n">
-        <v>0.00342222497387332</v>
+        <v>0.003425511282169029</v>
       </c>
     </row>
     <row r="25" customFormat="1" s="1">
@@ -3572,7 +3572,7 @@
         <v>1</v>
       </c>
       <c r="AJ25" t="n">
-        <v>28.9</v>
+        <v>28</v>
       </c>
       <c r="AK25" s="10" t="n">
         <v>47473</v>
@@ -3586,22 +3586,22 @@
         <v>494</v>
       </c>
       <c r="AY25" s="11" t="n">
-        <v>0.2493095995674254</v>
+        <v>0.2494769108931565</v>
       </c>
       <c r="AZ25" s="12" t="n">
-        <v>1.017301038062284</v>
+        <v>1.082142857142857</v>
       </c>
       <c r="BA25" s="8" t="n">
-        <v>2.901870034904349</v>
+        <v>2.899021196941307</v>
       </c>
       <c r="BB25" s="8" t="n">
-        <v>2.322778945994752</v>
+        <v>2.320187889561734</v>
       </c>
       <c r="BC25" s="8" t="n">
-        <v>3.273972602739726</v>
+        <v>3.271232876712329</v>
       </c>
       <c r="BD25" s="11" t="n">
-        <v>0.003446053710096503</v>
+        <v>0.003449440111217806</v>
       </c>
       <c r="BF25" s="16" t="n"/>
     </row>
@@ -3699,22 +3699,22 @@
         <v>1502</v>
       </c>
       <c r="AY26" s="11" t="n">
-        <v>68.59019802827143</v>
+        <v>69.18300653594773</v>
       </c>
       <c r="AZ26" s="12" t="n">
         <v>0.3966249999999998</v>
       </c>
       <c r="BA26" s="8" t="n">
-        <v>0.2986301369863013</v>
+        <v>0.2958904109589042</v>
       </c>
       <c r="BB26" s="8" t="n">
-        <v>0.004291267239460664</v>
+        <v>0.004215983691256503</v>
       </c>
       <c r="BC26" s="8" t="n">
-        <v>0.2712328767123288</v>
+        <v>0.2684931506849315</v>
       </c>
       <c r="BD26" s="11" t="n">
-        <v>0.0334862385321101</v>
+        <v>0.03379629629629629</v>
       </c>
     </row>
     <row r="27">
@@ -3808,22 +3808,22 @@
         <v>1484</v>
       </c>
       <c r="AY27" s="11" t="n">
-        <v>0.05417010269804687</v>
+        <v>0.05442058756680161</v>
       </c>
       <c r="AZ27" s="12" t="n">
         <v>0.542103365079365</v>
       </c>
       <c r="BA27" s="8" t="n">
-        <v>0.2931506849315069</v>
+        <v>0.2904109589041096</v>
       </c>
       <c r="BB27" s="8" t="n">
-        <v>0.2780866998420994</v>
+        <v>0.275422314708656</v>
       </c>
       <c r="BC27" s="8" t="n">
-        <v>0.2712328767123288</v>
+        <v>0.2684931506849315</v>
       </c>
       <c r="BD27" s="11" t="n">
-        <v>0.03411214953271028</v>
+        <v>0.03443396226415094</v>
       </c>
     </row>
     <row r="28" customFormat="1" s="1">
@@ -3921,7 +3921,7 @@
         <v>26.18372</v>
       </c>
       <c r="AJ28" t="n">
-        <v>12650</v>
+        <v>12760</v>
       </c>
       <c r="AK28" s="10" t="n">
         <v>46377</v>
@@ -3938,15 +3938,15 @@
         <v>1688</v>
       </c>
       <c r="AY28" s="11" t="n">
-        <v>-2.664974578356107</v>
+        <v>-2.689668646097396</v>
       </c>
       <c r="AZ28" s="12" t="n">
-        <v>0.05728412458498044</v>
+        <v>0.04816960626959266</v>
       </c>
       <c r="BA28" s="8" t="n"/>
       <c r="BB28" s="8" t="n"/>
       <c r="BC28" s="8" t="n">
-        <v>0.2712328767123288</v>
+        <v>0.2684931506849315</v>
       </c>
       <c r="BD28" s="11" t="n"/>
     </row>
@@ -4045,7 +4045,7 @@
         <v>115.1</v>
       </c>
       <c r="AJ29" t="n">
-        <v>17250</v>
+        <v>16920</v>
       </c>
       <c r="AK29" s="10" t="n">
         <v>47289</v>
@@ -4059,22 +4059,22 @@
         <v>1831</v>
       </c>
       <c r="AY29" s="11" t="n">
-        <v>-0.1574865595387808</v>
+        <v>-0.1576568795749231</v>
       </c>
       <c r="AZ29" s="12" t="n">
-        <v>0.2083831884057969</v>
+        <v>0.2319509456264774</v>
       </c>
       <c r="BA29" s="8" t="n">
-        <v>2.696952678367188</v>
+        <v>2.694243920063763</v>
       </c>
       <c r="BB29" s="8" t="n">
-        <v>3.201079708462323</v>
+        <v>3.198511217975105</v>
       </c>
       <c r="BC29" s="8" t="n">
-        <v>2.76986301369863</v>
+        <v>2.767123287671233</v>
       </c>
       <c r="BD29" s="11" t="n">
-        <v>0.003707888566311176</v>
+        <v>0.003711616429949422</v>
       </c>
     </row>
     <row r="30">
@@ -4189,22 +4189,22 @@
         <v>1974</v>
       </c>
       <c r="AY30" s="11" t="n">
-        <v>0.05530148308972638</v>
+        <v>0.05530080782280266</v>
       </c>
       <c r="AZ30" s="12" t="n">
         <v>0.6507586360555744</v>
       </c>
       <c r="BA30" s="8" t="n">
-        <v>2.643513020362766</v>
+        <v>2.640773444342202</v>
       </c>
       <c r="BB30" s="8" t="n">
-        <v>2.504983706289365</v>
+        <v>2.50238929484987</v>
       </c>
       <c r="BC30" s="8" t="n">
-        <v>2.76986301369863</v>
+        <v>2.767123287671233</v>
       </c>
       <c r="BD30" s="11" t="n">
-        <v>0.003782844995644361</v>
+        <v>0.003786769372974716</v>
       </c>
       <c r="BE30" s="1" t="n"/>
       <c r="BF30" s="1" t="n"/>
@@ -4286,7 +4286,7 @@
         <v>0.9284102</v>
       </c>
       <c r="AJ31" t="n">
-        <v>33.1</v>
+        <v>33</v>
       </c>
       <c r="AK31" s="10" t="n">
         <v>47133</v>
@@ -4303,22 +4303,22 @@
         <v>1369</v>
       </c>
       <c r="AY31" s="11" t="n">
-        <v>0.1168187008761466</v>
+        <v>0.1168786061321426</v>
       </c>
       <c r="AZ31" s="12" t="n">
-        <v>1.50754899939577</v>
+        <v>1.515147632727273</v>
       </c>
       <c r="BA31" s="8" t="n">
-        <v>2.178348445335936</v>
+        <v>2.175593510519608</v>
       </c>
       <c r="BB31" s="8" t="n">
-        <v>1.950494241927555</v>
+        <v>1.947922986951909</v>
       </c>
       <c r="BC31" s="8" t="n">
-        <v>2.342465753424658</v>
+        <v>2.33972602739726</v>
       </c>
       <c r="BD31" s="11" t="n">
-        <v>0.004590633799386416</v>
+        <v>0.004596446878356266</v>
       </c>
     </row>
     <row r="32">
@@ -4398,7 +4398,7 @@
         <v>430</v>
       </c>
       <c r="AJ32" t="n">
-        <v>69670</v>
+        <v>69000</v>
       </c>
       <c r="AK32" s="10" t="n">
         <v>46878</v>
@@ -4412,22 +4412,22 @@
         <v>1621</v>
       </c>
       <c r="AY32" s="11" t="n">
-        <v>-0.2728528560788701</v>
+        <v>-0.2732668611937489</v>
       </c>
       <c r="AZ32" s="12" t="n">
-        <v>0.1146548012056838</v>
+        <v>0.1254782608695653</v>
       </c>
       <c r="BA32" s="8" t="n">
-        <v>1.6412868371938</v>
+        <v>1.638562180032464</v>
       </c>
       <c r="BB32" s="8" t="n">
-        <v>2.257159160858675</v>
+        <v>2.254695833361893</v>
       </c>
       <c r="BC32" s="8" t="n">
-        <v>1.643835616438356</v>
+        <v>1.641095890410959</v>
       </c>
       <c r="BD32" s="11" t="n">
-        <v>0.006092780234012942</v>
+        <v>0.006102911517097187</v>
       </c>
     </row>
     <row r="33">
@@ -4521,22 +4521,22 @@
         <v>1949</v>
       </c>
       <c r="AY33" s="11" t="n">
-        <v>-0.1100844536724899</v>
+        <v>-0.1102222180299785</v>
       </c>
       <c r="AZ33" s="12" t="n">
         <v>0.005948460987831083</v>
       </c>
       <c r="BA33" s="8" t="n">
-        <v>2.678689892263281</v>
+        <v>2.675978096395653</v>
       </c>
       <c r="BB33" s="8" t="n">
-        <v>3.010049552811677</v>
+        <v>3.007467876384681</v>
       </c>
       <c r="BC33" s="8" t="n">
-        <v>2.76986301369863</v>
+        <v>2.767123287671233</v>
       </c>
       <c r="BD33" s="11" t="n">
-        <v>0.003733168228574152</v>
+        <v>0.003736951364986609</v>
       </c>
     </row>
     <row r="34">
@@ -4630,22 +4630,22 @@
         <v>634</v>
       </c>
       <c r="AY34" s="11" t="n">
-        <v>0.02975117298677777</v>
+        <v>0.02972745228127878</v>
       </c>
       <c r="AZ34" s="12" t="n">
         <v>0.29111266620014</v>
       </c>
       <c r="BA34" s="8" t="n">
-        <v>1.672607982568473</v>
+        <v>1.669869193105457</v>
       </c>
       <c r="BB34" s="8" t="n">
-        <v>1.624283639043691</v>
+        <v>1.621661333206176</v>
       </c>
       <c r="BC34" s="8" t="n">
-        <v>1.69041095890411</v>
+        <v>1.687671232876712</v>
       </c>
       <c r="BD34" s="11" t="n">
-        <v>0.005978687238263626</v>
+        <v>0.005988493015673275</v>
       </c>
     </row>
     <row r="35">

</xml_diff>